<commit_message>
Fill HSK1_parts_of_speech_6(251-300).xlsx with parts of speech
</commit_message>
<xml_diff>
--- a/HSK1_parts_of_speech_6(251-300).xlsx
+++ b/HSK1_parts_of_speech_6(251-300).xlsx
@@ -51,9 +51,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -601,6 +604,16 @@
           <t>где; куда уж мне</t>
         </is>
       </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>где?; куда? (вопросит. местоимение)</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>в иронич. отрицании — устойчивое выражение «куда уж мне»</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -627,6 +640,11 @@
           <t>где</t>
         </is>
       </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>где?; куда? (разг. вариант 哪里)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -653,6 +671,11 @@
           <t>какие</t>
         </is>
       </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>какие (вопросительное множественное)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -679,6 +702,16 @@
           <t>тот</t>
         </is>
       </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>тот, та, то</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="inlineStr">
+        <is>
+          <t>указательный элемент в составе 那个/那边</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -705,6 +738,11 @@
           <t>там, та сторона</t>
         </is>
       </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>та сторона; там (место-сущ.)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -731,6 +769,11 @@
           <t>там</t>
         </is>
       </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>там, то место (место-сущ.)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -757,6 +800,11 @@
           <t>там</t>
         </is>
       </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>там, то место (разг. вариант 那里)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -783,6 +831,11 @@
           <t>те</t>
         </is>
       </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>те (указательное множественное)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -809,6 +862,16 @@
           <t>молоко</t>
         </is>
       </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>молоко (разг., сокр. от 牛奶); грудь</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>кормить грудью</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -835,6 +898,11 @@
           <t>бабушка (со стороны отца)</t>
         </is>
       </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>бабушка (по отцовской линии)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -861,6 +929,21 @@
           <t>мужчина, мужской</t>
         </is>
       </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>мужчина; муж</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>мужской</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется (входит в состав слов: 男生, 男人)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -887,6 +970,11 @@
           <t>мальчик</t>
         </is>
       </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>мальчик</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -913,6 +1001,11 @@
           <t>(любимый) парень</t>
         </is>
       </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>парень (возлюбленный); друг-мужчина</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -939,6 +1032,11 @@
           <t>мужчина</t>
         </is>
       </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>мужчина (взрослый)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -965,6 +1063,11 @@
           <t>мальчик, юноша, ученик</t>
         </is>
       </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>ученик-юноша; мальчик (школ./разг.)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -991,6 +1094,16 @@
           <t>юг</t>
         </is>
       </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>юг, южная сторона</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется отдельно в разговорной речи (входит в 南边, 南瓜)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1017,6 +1130,11 @@
           <t>юг, южная сторона</t>
         </is>
       </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>юг, южная сторона</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1043,6 +1161,21 @@
           <t>сложный</t>
         </is>
       </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>беда, несчастье (难处)</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>трудный, сложный</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>трудно, с трудом (很难说)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1069,6 +1202,21 @@
           <t>фразовая частица</t>
         </is>
       </c>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>частица непрерывности действия / эллиптического вопроса («а я?»)</t>
+        </is>
+      </c>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>служебное слово</t>
+        </is>
+      </c>
+      <c r="Y20" s="2" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1095,6 +1243,11 @@
           <t>мочь, быть в состоянии</t>
         </is>
       </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>мочь, уметь; быть способным (модальный глагол)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1121,6 +1274,11 @@
           <t>ты</t>
         </is>
       </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>ты</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1147,6 +1305,11 @@
           <t>вы</t>
         </is>
       </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>вы (множественное)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1173,6 +1336,16 @@
           <t>год</t>
         </is>
       </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>год</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>для длительности времени и возраста (三年 = три года)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1199,6 +1372,11 @@
           <t>Вы</t>
         </is>
       </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>Вы (вежливая форма)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1225,6 +1403,11 @@
           <t>коровье молоко</t>
         </is>
       </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>коровье молоко</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1251,6 +1434,21 @@
           <t>женщина, женский</t>
         </is>
       </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>женщина; женский пол</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>женский</t>
+        </is>
+      </c>
+      <c r="Y27" s="2" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется (входит в состав слов: 女生, 女人)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1277,6 +1475,11 @@
           <t>дочь</t>
         </is>
       </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>дочь</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1303,6 +1506,11 @@
           <t>девушка</t>
         </is>
       </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>девочка, девушка</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1329,6 +1537,11 @@
           <t>(любимая) девушка, подруга</t>
         </is>
       </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>девушка (возлюбленная); подруга</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1355,6 +1568,11 @@
           <t>женщина</t>
         </is>
       </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>женщина</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1381,6 +1599,11 @@
           <t>девочка, девушка, ученица</t>
         </is>
       </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>ученица-девушка; девочка (школ./разг.)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1407,6 +1630,11 @@
           <t>рядом, поблизости</t>
         </is>
       </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>бок, сторона (в сочетании 旁边 — рядом, сбоку)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1433,6 +1661,11 @@
           <t>бегать</t>
         </is>
       </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>бегать; быстро двигаться (跑生意 — «крутиться, ездить по делам»)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1459,6 +1692,11 @@
           <t>друг</t>
         </is>
       </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>друг</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1485,6 +1723,16 @@
           <t>билет</t>
         </is>
       </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>билет</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>для билетов (一张票)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1511,6 +1759,11 @@
           <t>семь</t>
         </is>
       </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>семь (7)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1537,6 +1790,26 @@
           <t>подниматься, вставать</t>
         </is>
       </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>подниматься; вставать (как направ. дополнение)</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>для событий/волн (一起 = за один раз, 三起事故)</t>
+        </is>
+      </c>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>вместе, совместно (一起走)</t>
+        </is>
+      </c>
+      <c r="X38" s="2" t="inlineStr">
+        <is>
+          <t>полисемантичный глагол/наречие</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1563,6 +1836,16 @@
           <t>просыпаться, вставать с постели</t>
         </is>
       </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>вставать с постели, просыпаться</t>
+        </is>
+      </c>
+      <c r="X39" s="2" t="inlineStr">
+        <is>
+          <t>离合词 (разделяемое сочетание): 起了床</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1589,6 +1872,16 @@
           <t>вставать, начинаться</t>
         </is>
       </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>вставать; начинать(ся) (направ. компл. 起来)</t>
+        </is>
+      </c>
+      <c r="X40" s="2" t="inlineStr">
+        <is>
+          <t>служебная конструкция направления/начала действия</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1615,6 +1908,11 @@
           <t>автомобиль</t>
         </is>
       </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>автомобиль, машина</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1641,6 +1939,16 @@
           <t>перёд</t>
         </is>
       </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>перед, передняя часть</t>
+        </is>
+      </c>
+      <c r="X42" s="2" t="inlineStr">
+        <is>
+          <t>ориентир пространства; самостоятельно в речах ограничен (前边, 前天, 在…前)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1667,6 +1975,11 @@
           <t>передняя сторона</t>
         </is>
       </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>передняя сторона; впереди</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1693,6 +2006,16 @@
           <t>позавчера</t>
         </is>
       </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>позавчера (день перед вчера)</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>позавчера (как обстоятельство времени)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1719,6 +2042,11 @@
           <t>деньги</t>
         </is>
       </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>деньги</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1745,6 +2073,11 @@
           <t>кошелёк</t>
         </is>
       </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>кошелёк, бумажник</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1776,6 +2109,16 @@
           <t>да</t>
         </is>
       </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>просить; приглашать; пожалуйста (вежливая просьба)</t>
+        </is>
+      </c>
+      <c r="X47" s="2" t="inlineStr">
+        <is>
+          <t>вход в устойчивые формулы: 请进/请问/请坐</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1807,6 +2150,16 @@
           <t>да</t>
         </is>
       </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>брать отпуск/отгул; отпрашиваться</t>
+        </is>
+      </c>
+      <c r="X48" s="2" t="inlineStr">
+        <is>
+          <t>离合词: 请了一天假</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1838,6 +2191,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="X49" s="2" t="inlineStr">
+        <is>
+          <t>устойчивая пригласительная формула «Войдите!» (грамматическая конструкция)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1869,6 +2227,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="X50" s="2" t="inlineStr">
+        <is>
+          <t>устойчивая вводная формула «Разрешите спросить?» (грамматическая конструкция)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1898,6 +2261,11 @@
       <c r="J51" t="inlineStr">
         <is>
           <t>да</t>
+        </is>
+      </c>
+      <c r="X51" s="2" t="inlineStr">
+        <is>
+          <t>устойчивая формула гостеприимства «Пожалуйста, садитесь!» (грамматическая конструкция)</t>
         </is>
       </c>
     </row>

</xml_diff>